<commit_message>
v0.12.0: tabla de capacidad de trims con datos de fabricantes
- Cv, puerto y carrera típicos de globo y ángulo por familia de trim (mediana
  de datos publicados), trim reducido por restricciones en serie y alerta de
  coherencia ±10 %.
- Solapa 2: estilo de trim, sentido de flujo y característica independientes;
  Flow del actuador tomado del sentido; conversión de proyectos anteriores.
- Selección de trims especiales: verificación de capacidad y rangeabilidad.
- Materiales: «sin cavitación», temperatura de operación para corrosión y
  cloruros por encima de 100 °C en austeníticos.
- Ayuda ampliada (sentido de flujo, tabla de capacidad, Fγ), sentido de flujo
  en entregables, kit del workshop regenerado y pruebas de v0.12.0.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U4yJ7uLSXttFganqs6AWmH
</commit_message>
<xml_diff>
--- a/kit_workshop/Planilla_comparacion_workshop_N25.xlsx
+++ b/kit_workshop/Planilla_comparacion_workshop_N25.xlsx
@@ -780,7 +780,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>ΔP para flujo estrangulado (ΔP choked)</t>
+          <t>ΔP crítica de flujo estrangulado (ΔP choked)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -820,7 +820,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>ΔP para flujo estrangulado (ΔP choked)</t>
+          <t>ΔP crítica de flujo estrangulado (ΔP choked)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>ΔP para flujo estrangulado (ΔP choked)</t>
+          <t>ΔP crítica de flujo estrangulado (ΔP choked)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>20.6</v>
+        <v>57.1</v>
       </c>
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
@@ -1217,7 +1217,7 @@
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>33.1</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>52.9</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="n"/>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>ΔP para flujo estrangulado (ΔP choked)</t>
+          <t>ΔP crítica de flujo estrangulado (ΔP choked)</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>ΔP para flujo estrangulado (ΔP choked)</t>
+          <t>ΔP crítica de flujo estrangulado (ΔP choked)</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>ΔP para flujo estrangulado (ΔP choked)</t>
+          <t>ΔP crítica de flujo estrangulado (ΔP choked)</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -2933,7 +2933,7 @@
         </is>
       </c>
       <c r="E61" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F61" s="5" t="n"/>
       <c r="G61" s="5" t="n"/>
@@ -2973,7 +2973,7 @@
         </is>
       </c>
       <c r="E62" s="4" t="n">
-        <v>26</v>
+        <v>22.8</v>
       </c>
       <c r="F62" s="5" t="n"/>
       <c r="G62" s="5" t="n"/>
@@ -3013,7 +3013,7 @@
         </is>
       </c>
       <c r="E63" s="4" t="n">
-        <v>41.7</v>
+        <v>36.8</v>
       </c>
       <c r="F63" s="5" t="n"/>
       <c r="G63" s="5" t="n"/>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="D94" s="4" t="inlineStr"/>
       <c r="E94" s="4" t="n">
-        <v>5.773</v>
+        <v>5.78</v>
       </c>
       <c r="F94" s="5" t="n"/>
       <c r="G94" s="5" t="n"/>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="D95" s="4" t="inlineStr"/>
       <c r="E95" s="4" t="n">
-        <v>13.18</v>
+        <v>13.26</v>
       </c>
       <c r="F95" s="5" t="n"/>
       <c r="G95" s="5" t="n"/>
@@ -4273,7 +4273,7 @@
       </c>
       <c r="D96" s="4" t="inlineStr"/>
       <c r="E96" s="4" t="n">
-        <v>19.33</v>
+        <v>19.59</v>
       </c>
       <c r="F96" s="5" t="n"/>
       <c r="G96" s="5" t="n"/>
@@ -4304,7 +4304,7 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>ΔP para flujo estrangulado (ΔP choked)</t>
+          <t>ΔP crítica de flujo estrangulado (ΔP choked)</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -4313,7 +4313,7 @@
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>68.22</v>
+        <v>68.20999999999999</v>
       </c>
       <c r="F97" s="5" t="n"/>
       <c r="G97" s="5" t="n"/>
@@ -4344,7 +4344,7 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>ΔP para flujo estrangulado (ΔP choked)</t>
+          <t>ΔP crítica de flujo estrangulado (ΔP choked)</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
@@ -4353,7 +4353,7 @@
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>66.29000000000001</v>
+        <v>66.23999999999999</v>
       </c>
       <c r="F98" s="5" t="n"/>
       <c r="G98" s="5" t="n"/>
@@ -4384,7 +4384,7 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>ΔP para flujo estrangulado (ΔP choked)</t>
+          <t>ΔP crítica de flujo estrangulado (ΔP choked)</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -4393,7 +4393,7 @@
         </is>
       </c>
       <c r="E99" s="4" t="n">
-        <v>64.34999999999999</v>
+        <v>64.25</v>
       </c>
       <c r="F99" s="5" t="n"/>
       <c r="G99" s="5" t="n"/>
@@ -4429,7 +4429,7 @@
       </c>
       <c r="D100" s="4" t="inlineStr"/>
       <c r="E100" s="4" t="n">
-        <v>1</v>
+        <v>0.999</v>
       </c>
       <c r="F100" s="5" t="n"/>
       <c r="G100" s="5" t="n"/>
@@ -4465,7 +4465,7 @@
       </c>
       <c r="D101" s="4" t="inlineStr"/>
       <c r="E101" s="4" t="n">
-        <v>1</v>
+        <v>0.994</v>
       </c>
       <c r="F101" s="5" t="n"/>
       <c r="G101" s="5" t="n"/>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="D102" s="4" t="inlineStr"/>
       <c r="E102" s="4" t="n">
-        <v>0.999</v>
+        <v>0.987</v>
       </c>
       <c r="F102" s="5" t="n"/>
       <c r="G102" s="5" t="n"/>
@@ -4701,7 +4701,7 @@
         </is>
       </c>
       <c r="E107" s="4" t="n">
-        <v>15.5</v>
+        <v>19.8</v>
       </c>
       <c r="F107" s="5" t="n"/>
       <c r="G107" s="5" t="n"/>
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="E108" s="4" t="n">
-        <v>39.8</v>
+        <v>49.5</v>
       </c>
       <c r="F108" s="5" t="n"/>
       <c r="G108" s="5" t="n"/>
@@ -4781,7 +4781,7 @@
         </is>
       </c>
       <c r="E109" s="4" t="n">
-        <v>60</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="F109" s="5" t="n"/>
       <c r="G109" s="5" t="n"/>
@@ -4821,7 +4821,7 @@
         </is>
       </c>
       <c r="E110" s="4" t="n">
-        <v>72.09999999999999</v>
+        <v>77.8</v>
       </c>
       <c r="F110" s="5" t="n"/>
       <c r="G110" s="5" t="n"/>
@@ -4861,7 +4861,7 @@
         </is>
       </c>
       <c r="E111" s="4" t="n">
-        <v>77.09999999999999</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="F111" s="5" t="n"/>
       <c r="G111" s="5" t="n"/>
@@ -4901,7 +4901,7 @@
         </is>
       </c>
       <c r="E112" s="4" t="n">
-        <v>78.90000000000001</v>
+        <v>86.8</v>
       </c>
       <c r="F112" s="5" t="n"/>
       <c r="G112" s="5" t="n"/>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="D117" s="4" t="inlineStr"/>
       <c r="E117" s="4" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="F117" s="5" t="n"/>
       <c r="G117" s="5" t="n"/>
@@ -5117,7 +5117,7 @@
       </c>
       <c r="D118" s="4" t="inlineStr"/>
       <c r="E118" s="4" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="F118" s="5" t="n"/>
       <c r="G118" s="5" t="n"/>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="D119" s="4" t="inlineStr"/>
       <c r="E119" s="4" t="n">
-        <v>0.97</v>
+        <v>0.969</v>
       </c>
       <c r="F119" s="5" t="n"/>
       <c r="G119" s="5" t="n"/>
@@ -5189,7 +5189,7 @@
       </c>
       <c r="D120" s="4" t="inlineStr"/>
       <c r="E120" s="4" t="n">
-        <v>0.969</v>
+        <v>0.963</v>
       </c>
       <c r="F120" s="5" t="n"/>
       <c r="G120" s="5" t="n"/>
@@ -5225,7 +5225,7 @@
       </c>
       <c r="D121" s="4" t="inlineStr"/>
       <c r="E121" s="4" t="n">
-        <v>0.968</v>
+        <v>0.956</v>
       </c>
       <c r="F121" s="5" t="n"/>
       <c r="G121" s="5" t="n"/>
@@ -5265,7 +5265,7 @@
         </is>
       </c>
       <c r="E122" s="4" t="n">
-        <v>68.19</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="F122" s="5" t="n"/>
       <c r="G122" s="5" t="n"/>
@@ -5305,7 +5305,7 @@
         </is>
       </c>
       <c r="E123" s="4" t="n">
-        <v>66.26000000000001</v>
+        <v>66.22</v>
       </c>
       <c r="F123" s="5" t="n"/>
       <c r="G123" s="5" t="n"/>
@@ -5345,7 +5345,7 @@
         </is>
       </c>
       <c r="E124" s="4" t="n">
-        <v>64.33</v>
+        <v>64.23</v>
       </c>
       <c r="F124" s="5" t="n"/>
       <c r="G124" s="5" t="n"/>
@@ -5741,7 +5741,7 @@
       </c>
       <c r="D134" s="4" t="inlineStr"/>
       <c r="E134" s="4" t="n">
-        <v>214935</v>
+        <v>214811</v>
       </c>
       <c r="F134" s="5" t="n"/>
       <c r="G134" s="5" t="n"/>
@@ -5777,7 +5777,7 @@
       </c>
       <c r="D135" s="4" t="inlineStr"/>
       <c r="E135" s="4" t="n">
-        <v>320139</v>
+        <v>319169</v>
       </c>
       <c r="F135" s="5" t="n"/>
       <c r="G135" s="5" t="n"/>
@@ -5813,7 +5813,7 @@
       </c>
       <c r="D136" s="4" t="inlineStr"/>
       <c r="E136" s="4" t="n">
-        <v>381957</v>
+        <v>379457</v>
       </c>
       <c r="F136" s="5" t="n"/>
       <c r="G136" s="5" t="n"/>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Stellite 6 macizo (Co-Cr-W, fundido o forjado 6B) · 40 HRC (≈ 371 HB)</t>
+          <t>17-4PH H900 (40–47 HRC) · 44 HRC (≈ 411 HB)</t>
         </is>
       </c>
       <c r="D4" s="5" t="n"/>
@@ -6539,7 +6539,7 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Inconel 718 (N07718) envejecido · 38 HRC (≈ 353 HB)</t>
+          <t>17-4PH H1150D (≤ 33 HRC, NACE) · 30 HRC (≈ 286 HB)</t>
         </is>
       </c>
       <c r="D5" s="5" t="n"/>
@@ -6559,7 +6559,7 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Inconel 718 (N07718) envejecido · 38 HRC (≈ 353 HB)</t>
+          <t>17-4PH H1075 (≈ 33–38 HRC) · 35 HRC (≈ 327 HB)</t>
         </is>
       </c>
       <c r="D6" s="5" t="n"/>
@@ -6579,7 +6579,7 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Dúplex 2205 (S31803 / S32205) barra · 250 HB</t>
+          <t>Inoxidable 316 / 316L (A479, A276) · 150 HB</t>
         </is>
       </c>
       <c r="D7" s="5" t="n"/>
@@ -6799,7 +6799,7 @@
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Grafito flexible (anillos laminados + trenzas de carbono antiextrusión)</t>
+          <t>Grafito simple: cinta moldeada + trenzas de carbono antiextrusión</t>
         </is>
       </c>
       <c r="D18" s="5" t="n"/>

</xml_diff>

<commit_message>
v0.13.0: trims por tipo, guía y nivel; multietapa multiorificio para gas
- Desplegables en orden: tipo de trim (obturador / jaula), guía y obturador, o jaula según fluido,
  nivel o etapas individual con su mitigación, sentido, balance y característica permitida.
- Jaula multietapa multiorificio para gas (2, 3 y 4 etapas) con ruido de la última etapa.
- Obturador en V, microcaudal (hasta 2"), disco plano, característica parabólica modificada.
- Migración de proyectos v0.11 y v0.12; kit del workshop regenerado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U4yJ7uLSXttFganqs6AWmH
</commit_message>
<xml_diff>
--- a/kit_workshop/Planilla_comparacion_workshop_N25.xlsx
+++ b/kit_workshop/Planilla_comparacion_workshop_N25.xlsx
@@ -4201,7 +4201,7 @@
       </c>
       <c r="D94" s="4" t="inlineStr"/>
       <c r="E94" s="4" t="n">
-        <v>5.78</v>
+        <v>6.028</v>
       </c>
       <c r="F94" s="5" t="n"/>
       <c r="G94" s="5" t="n"/>
@@ -4237,7 +4237,7 @@
       </c>
       <c r="D95" s="4" t="inlineStr"/>
       <c r="E95" s="4" t="n">
-        <v>13.26</v>
+        <v>13.83</v>
       </c>
       <c r="F95" s="5" t="n"/>
       <c r="G95" s="5" t="n"/>
@@ -4273,7 +4273,7 @@
       </c>
       <c r="D96" s="4" t="inlineStr"/>
       <c r="E96" s="4" t="n">
-        <v>19.59</v>
+        <v>20.43</v>
       </c>
       <c r="F96" s="5" t="n"/>
       <c r="G96" s="5" t="n"/>
@@ -4313,7 +4313,7 @@
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>68.20999999999999</v>
+        <v>62.71</v>
       </c>
       <c r="F97" s="5" t="n"/>
       <c r="G97" s="5" t="n"/>
@@ -4353,7 +4353,7 @@
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>66.23999999999999</v>
+        <v>60.96</v>
       </c>
       <c r="F98" s="5" t="n"/>
       <c r="G98" s="5" t="n"/>
@@ -4393,7 +4393,7 @@
         </is>
       </c>
       <c r="E99" s="4" t="n">
-        <v>64.25</v>
+        <v>59.2</v>
       </c>
       <c r="F99" s="5" t="n"/>
       <c r="G99" s="5" t="n"/>
@@ -4465,7 +4465,7 @@
       </c>
       <c r="D101" s="4" t="inlineStr"/>
       <c r="E101" s="4" t="n">
-        <v>0.994</v>
+        <v>0.993</v>
       </c>
       <c r="F101" s="5" t="n"/>
       <c r="G101" s="5" t="n"/>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="D102" s="4" t="inlineStr"/>
       <c r="E102" s="4" t="n">
-        <v>0.987</v>
+        <v>0.986</v>
       </c>
       <c r="F102" s="5" t="n"/>
       <c r="G102" s="5" t="n"/>
@@ -4701,7 +4701,7 @@
         </is>
       </c>
       <c r="E107" s="4" t="n">
-        <v>19.8</v>
+        <v>8.24</v>
       </c>
       <c r="F107" s="5" t="n"/>
       <c r="G107" s="5" t="n"/>
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="E108" s="4" t="n">
-        <v>49.5</v>
+        <v>28.1</v>
       </c>
       <c r="F108" s="5" t="n"/>
       <c r="G108" s="5" t="n"/>
@@ -4781,7 +4781,7 @@
         </is>
       </c>
       <c r="E109" s="4" t="n">
-        <v>74.59999999999999</v>
+        <v>45</v>
       </c>
       <c r="F109" s="5" t="n"/>
       <c r="G109" s="5" t="n"/>
@@ -4821,7 +4821,7 @@
         </is>
       </c>
       <c r="E110" s="4" t="n">
-        <v>77.8</v>
+        <v>86.3</v>
       </c>
       <c r="F110" s="5" t="n"/>
       <c r="G110" s="5" t="n"/>
@@ -4861,7 +4861,7 @@
         </is>
       </c>
       <c r="E111" s="4" t="n">
-        <v>83.90000000000001</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="F111" s="5" t="n"/>
       <c r="G111" s="5" t="n"/>
@@ -4901,7 +4901,7 @@
         </is>
       </c>
       <c r="E112" s="4" t="n">
-        <v>86.8</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="F112" s="5" t="n"/>
       <c r="G112" s="5" t="n"/>
@@ -5045,7 +5045,7 @@
       </c>
       <c r="D116" s="4" t="inlineStr"/>
       <c r="E116" s="4" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.504</v>
       </c>
       <c r="F116" s="5" t="n"/>
       <c r="G116" s="5" t="n"/>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="D117" s="4" t="inlineStr"/>
       <c r="E117" s="4" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.459</v>
       </c>
       <c r="F117" s="5" t="n"/>
       <c r="G117" s="5" t="n"/>
@@ -5117,7 +5117,7 @@
       </c>
       <c r="D118" s="4" t="inlineStr"/>
       <c r="E118" s="4" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.437</v>
       </c>
       <c r="F118" s="5" t="n"/>
       <c r="G118" s="5" t="n"/>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="D119" s="4" t="inlineStr"/>
       <c r="E119" s="4" t="n">
-        <v>0.969</v>
+        <v>0.929</v>
       </c>
       <c r="F119" s="5" t="n"/>
       <c r="G119" s="5" t="n"/>
@@ -5189,7 +5189,7 @@
       </c>
       <c r="D120" s="4" t="inlineStr"/>
       <c r="E120" s="4" t="n">
-        <v>0.963</v>
+        <v>0.924</v>
       </c>
       <c r="F120" s="5" t="n"/>
       <c r="G120" s="5" t="n"/>
@@ -5225,7 +5225,7 @@
       </c>
       <c r="D121" s="4" t="inlineStr"/>
       <c r="E121" s="4" t="n">
-        <v>0.956</v>
+        <v>0.916</v>
       </c>
       <c r="F121" s="5" t="n"/>
       <c r="G121" s="5" t="n"/>
@@ -5265,7 +5265,7 @@
         </is>
       </c>
       <c r="E122" s="4" t="n">
-        <v>68.18000000000001</v>
+        <v>61.61</v>
       </c>
       <c r="F122" s="5" t="n"/>
       <c r="G122" s="5" t="n"/>
@@ -5305,7 +5305,7 @@
         </is>
       </c>
       <c r="E123" s="4" t="n">
-        <v>66.22</v>
+        <v>59.91</v>
       </c>
       <c r="F123" s="5" t="n"/>
       <c r="G123" s="5" t="n"/>
@@ -5345,7 +5345,7 @@
         </is>
       </c>
       <c r="E124" s="4" t="n">
-        <v>64.23</v>
+        <v>58.21</v>
       </c>
       <c r="F124" s="5" t="n"/>
       <c r="G124" s="5" t="n"/>
@@ -5741,7 +5741,7 @@
       </c>
       <c r="D134" s="4" t="inlineStr"/>
       <c r="E134" s="4" t="n">
-        <v>214811</v>
+        <v>306873</v>
       </c>
       <c r="F134" s="5" t="n"/>
       <c r="G134" s="5" t="n"/>
@@ -5777,7 +5777,7 @@
       </c>
       <c r="D135" s="4" t="inlineStr"/>
       <c r="E135" s="4" t="n">
-        <v>319169</v>
+        <v>455956</v>
       </c>
       <c r="F135" s="5" t="n"/>
       <c r="G135" s="5" t="n"/>
@@ -5813,7 +5813,7 @@
       </c>
       <c r="D136" s="4" t="inlineStr"/>
       <c r="E136" s="4" t="n">
-        <v>379457</v>
+        <v>542082</v>
       </c>
       <c r="F136" s="5" t="n"/>
       <c r="G136" s="5" t="n"/>

</xml_diff>

<commit_message>
v0.13.4: área de salida de la válvula automática (tabla ASME B36 completa)
- tuberias: tabla ASME B36.10M / B36.19M de 1/8" a 80" (44 tamaños, 379
  combinaciones NPS-cédula), área interior π/4·DI² y área de salida de la
  válvula con el NPS de la válvula y la cédula de salida; si la cédula no
  existe para ese tamaño se usa STD con aviso.
- Fila «Área de salida de la válvula» con desplegable Automático / Manual,
  visible también en líquidos; el área gobierna la velocidad de salida
  (líquido, bifásico y gas) y el ruido aerodinámico IEC 60534-8-3.
- Memoria y hoja de datos muestran el área y su origen.
- Proyectos anteriores con área cargada quedan en Manual.
- Se quita el botón «Nuevo cálculo» de la v0.13.3 por decisión de Andrea
  (revert de 0817fce); la base de esta versión es la 0.13.2.
- Kit del workshop regenerado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U4yJ7uLSXttFganqs6AWmH
</commit_message>
<xml_diff>
--- a/kit_workshop/Planilla_comparacion_workshop_N25.xlsx
+++ b/kit_workshop/Planilla_comparacion_workshop_N25.xlsx
@@ -3053,7 +3053,7 @@
         </is>
       </c>
       <c r="E64" s="4" t="n">
-        <v>97.5</v>
+        <v>97.7</v>
       </c>
       <c r="F64" s="5" t="n"/>
       <c r="G64" s="5" t="n"/>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="D67" s="4" t="inlineStr"/>
       <c r="E67" s="4" t="n">
-        <v>0.111</v>
+        <v>0.106</v>
       </c>
       <c r="F67" s="5" t="n"/>
       <c r="G67" s="5" t="n"/>
@@ -3205,7 +3205,7 @@
       </c>
       <c r="D68" s="4" t="inlineStr"/>
       <c r="E68" s="4" t="n">
-        <v>0.166</v>
+        <v>0.159</v>
       </c>
       <c r="F68" s="5" t="n"/>
       <c r="G68" s="5" t="n"/>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="D69" s="4" t="inlineStr"/>
       <c r="E69" s="4" t="n">
-        <v>0.25</v>
+        <v>0.239</v>
       </c>
       <c r="F69" s="5" t="n"/>
       <c r="G69" s="5" t="n"/>
@@ -3281,7 +3281,7 @@
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>68.2</v>
+        <v>65.2</v>
       </c>
       <c r="F70" s="5" t="n"/>
       <c r="G70" s="5" t="n"/>
@@ -3321,7 +3321,7 @@
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>102</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="F71" s="5" t="n"/>
       <c r="G71" s="5" t="n"/>
@@ -3361,7 +3361,7 @@
         </is>
       </c>
       <c r="E72" s="4" t="n">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="F72" s="5" t="n"/>
       <c r="G72" s="5" t="n"/>

</xml_diff>